<commit_message>
update clusterGA code to match with the paper
</commit_message>
<xml_diff>
--- a/results/cluster_ga/UAVs3_GRID13/revenue/UAVs3_GRID13_Greedy.xlsx
+++ b/results/cluster_ga/UAVs3_GRID13/revenue/UAVs3_GRID13_Greedy.xlsx
@@ -642,13 +642,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.74502081770338</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.00584191586371</v>
-      </c>
-      <c r="D2" t="n">
-        <v>39.15540347000338</v>
+        <v>24.41193106929261</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.91719270494497</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.38695220645081</v>
       </c>
     </row>
   </sheetData>
@@ -692,13 +692,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.5409352808537</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.77164516313428</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.99323936650039</v>
+        <v>26.39072429262812</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.80591307656732</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.46639778637776</v>
       </c>
     </row>
   </sheetData>
@@ -742,13 +742,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>33.766730471054</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.90683852044639</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.78903395811609</v>
+        <v>19.70876144890668</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.97895144161064</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.72146366470049</v>
       </c>
     </row>
   </sheetData>
@@ -792,13 +792,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.39288805582899</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.52106038262849</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.6317364583287</v>
+        <v>21.02275075691368</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.05873015190059</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.41589139084699</v>
       </c>
     </row>
   </sheetData>
@@ -842,13 +842,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.97739872353332</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.0061631590617</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.26321012009231</v>
+        <v>22.94684013011025</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.34615271942581</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.18051770559967</v>
       </c>
     </row>
   </sheetData>
@@ -892,13 +892,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.88712868545984</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.61145386608971</v>
-      </c>
-      <c r="D2" t="n">
-        <v>44.57635729965533</v>
+        <v>25.94277236700007</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.99032621931648</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.77628524231944</v>
       </c>
     </row>
   </sheetData>
@@ -942,13 +942,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>17.31334418865518</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.45872811235393</v>
-      </c>
-      <c r="D2" t="n">
-        <v>34.69564295165014</v>
+        <v>19.00414374952524</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.74809059079432</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.27623621817886</v>
       </c>
     </row>
   </sheetData>
@@ -992,13 +992,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.44990535924939</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.0227878877521</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.82132692293983</v>
+        <v>25.85263283285062</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.71522447067131</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.02287896797837</v>
       </c>
     </row>
   </sheetData>
@@ -1042,13 +1042,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.2979666246661</v>
-      </c>
-      <c r="C2" t="n">
-        <v>34.01681951282242</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.42182889022934</v>
+        <v>27.32186374844024</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.52009816276944</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.53639908356001</v>
       </c>
     </row>
   </sheetData>
@@ -1092,13 +1092,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.31654718908261</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.73226718957623</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.54960095028495</v>
+        <v>20.89679877881625</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.6111879265847</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.86948854289238</v>
       </c>
     </row>
   </sheetData>
@@ -1142,13 +1142,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.50691434819468</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.08276419607105</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.21756735015666</v>
+        <v>22.09172828864536</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.23560367117592</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.77713900525124</v>
       </c>
     </row>
   </sheetData>
@@ -1192,13 +1192,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>35.95944066503571</v>
-      </c>
-      <c r="C2" t="n">
-        <v>29.73217289756355</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.16521033477764</v>
+        <v>27.63872172453603</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.92436533772203</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.35519913774049</v>
       </c>
     </row>
   </sheetData>
@@ -1242,13 +1242,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.3422663643955</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.68430793015799</v>
-      </c>
-      <c r="D2" t="n">
-        <v>35.14948561767331</v>
+        <v>20.5667437839385</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.8241733514425</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.31932335656823</v>
       </c>
     </row>
   </sheetData>
@@ -1292,13 +1292,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.01588792387204</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.42806277440786</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.30735573390609</v>
+        <v>20.13707272973053</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.36294012461794</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.92926155460204</v>
       </c>
     </row>
   </sheetData>
@@ -1342,13 +1342,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.64925399659345</v>
-      </c>
-      <c r="C2" t="n">
-        <v>31.8087806179975</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.14447537694776</v>
+        <v>17.86608600286051</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.95937457868608</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.50880334370353</v>
       </c>
     </row>
   </sheetData>
@@ -1392,13 +1392,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>22.64250435103703</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.44093144325945</v>
-      </c>
-      <c r="D2" t="n">
-        <v>34.70027692075946</v>
+        <v>20.39087685624306</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.71023904236861</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.70274452069858</v>
       </c>
     </row>
   </sheetData>
@@ -1442,13 +1442,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>34.16436687237122</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.31071219982051</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.59896623766496</v>
+        <v>25.12540986683749</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.61864735655447</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.41602481016652</v>
       </c>
     </row>
   </sheetData>
@@ -1492,13 +1492,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.79485613395953</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.19799137020305</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.61748807416949</v>
+        <v>18.14081511655589</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.06327408355864</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.33349672177718</v>
       </c>
     </row>
   </sheetData>
@@ -1542,13 +1542,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.56113731077717</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.6348419047252</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.39503703876958</v>
+        <v>23.3145656909482</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.58387320879106</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.80854328051056</v>
       </c>
     </row>
   </sheetData>
@@ -1592,13 +1592,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.93343913555355</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.60332032834264</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.82696559626786</v>
+        <v>19.15469932302922</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24.83373157721208</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.50261960207982</v>
       </c>
     </row>
   </sheetData>
@@ -1642,13 +1642,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.67958583792092</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.76656430368989</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.09408697711469</v>
+        <v>16.62973060989766</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.06890922811543</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.16485171024601</v>
       </c>
     </row>
   </sheetData>
@@ -1692,13 +1692,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.92613209629851</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.25270860103502</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.00522089914634</v>
+        <v>16.23954511386913</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.5742987017859</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.80343934708014</v>
       </c>
     </row>
   </sheetData>
@@ -1742,13 +1742,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.13995937277194</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.2367164624049</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.79294184187082</v>
+        <v>23.67656554860938</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.99483071983768</v>
+      </c>
+      <c r="D2" t="n">
+        <v>30.62273893318902</v>
       </c>
     </row>
   </sheetData>
@@ -1792,13 +1792,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.47706601552773</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.28861081487083</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.2116200015935</v>
+        <v>17.01673386973482</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.8174384769817</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.18124855162598</v>
       </c>
     </row>
   </sheetData>
@@ -1842,13 +1842,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>23.60073872321084</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.27139167645984</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.24701373639218</v>
+        <v>19.35792855106704</v>
+      </c>
+      <c r="C2" t="n">
+        <v>16.31249296771107</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.99055509102438</v>
       </c>
     </row>
   </sheetData>
@@ -1892,13 +1892,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.7913896208435</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.3299700939179</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.21471513898427</v>
+        <v>24.2239458163876</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.55081219359229</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.34493612428491</v>
       </c>
     </row>
   </sheetData>
@@ -1942,13 +1942,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.68314677769287</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.50261368260747</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.24558922917432</v>
+        <v>18.36237943214339</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.16960557319831</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.11972506930656</v>
       </c>
     </row>
   </sheetData>
@@ -1992,13 +1992,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>20.51219417488901</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.55618956330333</v>
-      </c>
-      <c r="D2" t="n">
-        <v>34.99265873549361</v>
+        <v>20.66763422392294</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24.86826931621442</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.37803937486931</v>
       </c>
     </row>
   </sheetData>
@@ -2042,13 +2042,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.85108209863836</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.27559942931564</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.07366528782238</v>
+        <v>16.96726892414768</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.66297079486515</v>
+      </c>
+      <c r="D2" t="n">
+        <v>30.1527686794008</v>
       </c>
     </row>
   </sheetData>
@@ -2092,13 +2092,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>33.88714808285309</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.3746731971448</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.31931822536041</v>
+        <v>18.18162390218386</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.95708601611238</v>
+      </c>
+      <c r="D2" t="n">
+        <v>29.45387001258018</v>
       </c>
     </row>
   </sheetData>
@@ -2142,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.43708233264429</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.05286004466709</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.26588801193076</v>
+        <v>23.26752843983038</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.24048573039883</v>
+      </c>
+      <c r="D2" t="n">
+        <v>18.75312534988734</v>
       </c>
     </row>
   </sheetData>
@@ -2192,13 +2192,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.48623081142422</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.44742128998976</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.02300714629679</v>
+        <v>17.84431431482252</v>
+      </c>
+      <c r="C2" t="n">
+        <v>30.54798859020195</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.26725262597428</v>
       </c>
     </row>
   </sheetData>
@@ -2242,13 +2242,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.65089628343836</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.2988526102226</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.01057220018551</v>
+        <v>18.84525695677398</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24.67107707334098</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.7143481380865</v>
       </c>
     </row>
   </sheetData>
@@ -2292,13 +2292,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>33.38356471319422</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.51512223292893</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.61565443989069</v>
+        <v>20.4960684236918</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.23541065976606</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.03055885197515</v>
       </c>
     </row>
   </sheetData>
@@ -2342,13 +2342,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.91266759453027</v>
-      </c>
-      <c r="C2" t="n">
-        <v>30.07682335714456</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.06460456113445</v>
+        <v>21.03064761734976</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.53773504869014</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.35774893878314</v>
       </c>
     </row>
   </sheetData>
@@ -2392,13 +2392,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.38942990319748</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.8638766280949</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.18020754900619</v>
+        <v>18.04923218172918</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.58220908348681</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.4220985801221</v>
       </c>
     </row>
   </sheetData>
@@ -2442,13 +2442,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>33.73758140049727</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.3232448322464</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.11013044379186</v>
+        <v>24.28972647555591</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.69922851744026</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.0008348296275</v>
       </c>
     </row>
   </sheetData>
@@ -2492,13 +2492,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.2128587973432</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.57939289796248</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.16239228194458</v>
+        <v>22.55853050258136</v>
+      </c>
+      <c r="C2" t="n">
+        <v>15.41092890222228</v>
+      </c>
+      <c r="D2" t="n">
+        <v>19.94442719339446</v>
       </c>
     </row>
   </sheetData>
@@ -2542,13 +2542,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.47421279510973</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.02968778100254</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.89155446459784</v>
+        <v>17.60945751088596</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.32067561318122</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.05147762855179</v>
       </c>
     </row>
   </sheetData>
@@ -2592,13 +2592,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.40226771707079</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.70307980510227</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.66279798284786</v>
+        <v>21.93810178754653</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.1095825082112</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.3682075680291</v>
       </c>
     </row>
   </sheetData>
@@ -2642,13 +2642,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.28637011833866</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.74720521016359</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.81471380407578</v>
+        <v>27.56530696363423</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.07694282193201</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.53411982175519</v>
       </c>
     </row>
   </sheetData>
@@ -2692,13 +2692,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.88776765915236</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.49964786145236</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.24014692337992</v>
+        <v>21.52211984497083</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.28280234623452</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.76629188101584</v>
       </c>
     </row>
   </sheetData>
@@ -2742,13 +2742,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.39907144822501</v>
-      </c>
-      <c r="C2" t="n">
-        <v>31.50612737473913</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.16796841424725</v>
+        <v>17.46034682890849</v>
+      </c>
+      <c r="C2" t="n">
+        <v>29.60554217859026</v>
+      </c>
+      <c r="D2" t="n">
+        <v>31.98149279079415</v>
       </c>
     </row>
   </sheetData>
@@ -2792,13 +2792,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>35.34852615044205</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.13435708484787</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.18871218837189</v>
+        <v>18.53680663608451</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.74544848633752</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.75822445402864</v>
       </c>
     </row>
   </sheetData>
@@ -2842,13 +2842,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.83245405379334</v>
-      </c>
-      <c r="C2" t="n">
-        <v>31.97945227192306</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.51736735331372</v>
+        <v>19.2940129397504</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24.64869206841396</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.8743329883888</v>
       </c>
     </row>
   </sheetData>
@@ -2892,13 +2892,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.49208964467499</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.69487777450192</v>
-      </c>
-      <c r="D2" t="n">
-        <v>33.16829767631</v>
+        <v>22.21513953173164</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.93157141700065</v>
+      </c>
+      <c r="D2" t="n">
+        <v>29.6516858948799</v>
       </c>
     </row>
   </sheetData>
@@ -2942,13 +2942,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.76255573994925</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.12597904779533</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.63882050103252</v>
+        <v>23.44842184716863</v>
+      </c>
+      <c r="C2" t="n">
+        <v>15.83626362360605</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.09901392416693</v>
       </c>
     </row>
   </sheetData>
@@ -2992,13 +2992,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.50792929804735</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.56090814074126</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.05123574494049</v>
+        <v>21.44368546130463</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24.64757763601472</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.34637650316832</v>
       </c>
     </row>
   </sheetData>
@@ -3042,13 +3042,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.82185198641799</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.45356521778755</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.14569030314443</v>
+        <v>18.77913605293671</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.21072179144486</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.23468491661599</v>
       </c>
     </row>
   </sheetData>
@@ -3092,13 +3092,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.35928984903407</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.02315334752287</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.25320794296617</v>
+        <v>20.44824756527308</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.06603952781633</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.46820076819491</v>
       </c>
     </row>
   </sheetData>
@@ -3142,13 +3142,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.36249066635673</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.17845929038437</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.27195059099135</v>
+        <v>24.67400624811153</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.25441735472043</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.19901060495442</v>
       </c>
     </row>
   </sheetData>
@@ -3192,13 +3192,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.11315560430765</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.97538476397806</v>
-      </c>
-      <c r="D2" t="n">
-        <v>34.09639958000476</v>
+        <v>19.42419684833695</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.49968257719637</v>
+      </c>
+      <c r="D2" t="n">
+        <v>19.68903518870193</v>
       </c>
     </row>
   </sheetData>
@@ -3242,13 +3242,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>23.65332856638072</v>
-      </c>
-      <c r="C2" t="n">
-        <v>30.39452266423224</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.10000780110029</v>
+        <v>22.56350172914719</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.65842080856426</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.29690277105238</v>
       </c>
     </row>
   </sheetData>
@@ -3292,13 +3292,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.60450654482359</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.44614569500601</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.33226320323581</v>
+        <v>26.38924339996366</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.87212579371048</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.32023853023544</v>
       </c>
     </row>
   </sheetData>
@@ -3342,13 +3342,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.01300601691825</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.03125433942662</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.09045388810773</v>
+        <v>18.97495078381741</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.70177778707464</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.43744951583382</v>
       </c>
     </row>
   </sheetData>
@@ -3392,13 +3392,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.10950253953569</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.45066786094034</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.27100603342128</v>
+        <v>21.45951752837786</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.36632642536232</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.33486288084147</v>
       </c>
     </row>
   </sheetData>
@@ -3442,13 +3442,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.56034650020127</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.10616802428082</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.25348224944623</v>
+        <v>21.61401862046718</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.81523692648469</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.03448740188119</v>
       </c>
     </row>
   </sheetData>
@@ -3492,13 +3492,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.11682829806787</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.67085907026237</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.18019819141083</v>
+        <v>21.78576351593854</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24.84171749391091</v>
+      </c>
+      <c r="D2" t="n">
+        <v>29.26650178912314</v>
       </c>
     </row>
   </sheetData>
@@ -3542,13 +3542,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.16867610584845</v>
-      </c>
-      <c r="C2" t="n">
-        <v>35.38817985507696</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.90536206485579</v>
+        <v>18.70378426499574</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.33691600641928</v>
+      </c>
+      <c r="D2" t="n">
+        <v>32.92050925999973</v>
       </c>
     </row>
   </sheetData>
@@ -3592,13 +3592,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.78181720298786</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.51931039420756</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.65258877952407</v>
+        <v>24.59278774499576</v>
+      </c>
+      <c r="C2" t="n">
+        <v>17.01106510086587</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.48058920248519</v>
       </c>
     </row>
   </sheetData>
@@ -3642,13 +3642,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.81486158842916</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.96337093073547</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.90002831589453</v>
+        <v>19.09043854554242</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.65066325482727</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.69680900840887</v>
       </c>
     </row>
   </sheetData>
@@ -3692,13 +3692,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>22.72840043137299</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.52809279424521</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.21038940359906</v>
+        <v>17.95762717997647</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.04982844017348</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.35274147293192</v>
       </c>
     </row>
   </sheetData>
@@ -3742,13 +3742,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.50751996098155</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.56520798349186</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.86326155415856</v>
+        <v>25.95714499704781</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.49177886352149</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.57004287111903</v>
       </c>
     </row>
   </sheetData>
@@ -3792,13 +3792,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.23827679979077</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.05833964633681</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.4099823976256</v>
+        <v>19.86555036188364</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.22678807547425</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.95501092626606</v>
       </c>
     </row>
   </sheetData>
@@ -3842,13 +3842,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.44709796890797</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.46436981860043</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.78542138480404</v>
+        <v>18.04056905986402</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24.80942286365754</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.82476002183327</v>
       </c>
     </row>
   </sheetData>
@@ -3892,13 +3892,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.6431699663916</v>
-      </c>
-      <c r="C2" t="n">
-        <v>29.51028743174671</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.96385201170354</v>
+        <v>26.12965443959055</v>
+      </c>
+      <c r="C2" t="n">
+        <v>16.68987863851615</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.18049672029077</v>
       </c>
     </row>
   </sheetData>
@@ -3942,13 +3942,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.70960377274469</v>
-      </c>
-      <c r="C2" t="n">
-        <v>37.07977657038514</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.66796275147769</v>
+        <v>20.43309257549689</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.85728492283579</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.94411464425751</v>
       </c>
     </row>
   </sheetData>
@@ -3992,13 +3992,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>37.24307721477866</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.27650116974506</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.48792945898501</v>
+        <v>21.88780055260479</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.61431295232833</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.62917276761532</v>
       </c>
     </row>
   </sheetData>
@@ -4042,13 +4042,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>36.16314442815045</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.09106977120194</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.51164489422285</v>
+        <v>23.19345823408132</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24.01998184054873</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.53147106132513</v>
       </c>
     </row>
   </sheetData>
@@ -4092,13 +4092,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.29672913987452</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.10248317403946</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.06206430926031</v>
+        <v>21.89661343526062</v>
+      </c>
+      <c r="C2" t="n">
+        <v>15.82587469951517</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.33598720322962</v>
       </c>
     </row>
   </sheetData>
@@ -4142,13 +4142,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.76785585863886</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.63220132299359</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.65505720630234</v>
+        <v>17.39917315918827</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.40593679079122</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.96034224713489</v>
       </c>
     </row>
   </sheetData>
@@ -4192,13 +4192,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.92861638304133</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.33902582272414</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.03338844526447</v>
+        <v>25.11006877200602</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.16085722352696</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.58758017280402</v>
       </c>
     </row>
   </sheetData>
@@ -4242,13 +4242,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.21721734674357</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.2649047324988</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.20759099737668</v>
+        <v>25.48667929589364</v>
+      </c>
+      <c r="C2" t="n">
+        <v>17.62135186967467</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.55624081572758</v>
       </c>
     </row>
   </sheetData>
@@ -4292,13 +4292,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.35514890049568</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.12565233452127</v>
-      </c>
-      <c r="D2" t="n">
-        <v>33.06006323436851</v>
+        <v>17.71459838547401</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24.4647105091812</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.43926113029865</v>
       </c>
     </row>
   </sheetData>
@@ -4342,13 +4342,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>33.60686143160655</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.51907063042826</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.34738853360872</v>
+        <v>24.10721392847265</v>
+      </c>
+      <c r="C2" t="n">
+        <v>28.83685840374489</v>
+      </c>
+      <c r="D2" t="n">
+        <v>19.83987801412736</v>
       </c>
     </row>
   </sheetData>
@@ -4392,13 +4392,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>21.32342932954371</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.16913342824716</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.53996875150363</v>
+        <v>17.66463894181173</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.57685998188458</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.81680705904997</v>
       </c>
     </row>
   </sheetData>
@@ -4442,13 +4442,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.5591942445246</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.01324829392547</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.46976369998896</v>
+        <v>20.37036866718558</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.36657809970418</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.97073517205835</v>
       </c>
     </row>
   </sheetData>
@@ -4492,13 +4492,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.99540148718498</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.33892089153401</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.02228707559464</v>
+        <v>19.64217312134599</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.15050009551107</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.41628398078555</v>
       </c>
     </row>
   </sheetData>
@@ -4542,13 +4542,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>21.16421665220624</v>
-      </c>
-      <c r="C2" t="n">
-        <v>39.54319563423561</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.88038706960233</v>
+        <v>18.46417736837623</v>
+      </c>
+      <c r="C2" t="n">
+        <v>28.39660537499277</v>
+      </c>
+      <c r="D2" t="n">
+        <v>30.03445878636449</v>
       </c>
     </row>
   </sheetData>
@@ -4592,13 +4592,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.56667881478189</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.37864292838509</v>
-      </c>
-      <c r="D2" t="n">
-        <v>40.91602179128753</v>
+        <v>19.98976700609475</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.20008758923888</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.42524613516096</v>
       </c>
     </row>
   </sheetData>
@@ -4642,13 +4642,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.90394395046667</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.3485669632909</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.97677489574351</v>
+        <v>23.10992471444893</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.05508978484108</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.23248460090994</v>
       </c>
     </row>
   </sheetData>
@@ -4692,13 +4692,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.66754427951156</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.75663138182476</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.42645840768514</v>
+        <v>17.46915462406644</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.95379913898936</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.13375779926783</v>
       </c>
     </row>
   </sheetData>
@@ -4742,13 +4742,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.35357196555821</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.46994256603974</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.59882797484341</v>
+        <v>17.52942255752297</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.30690801522296</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.80614039903159</v>
       </c>
     </row>
   </sheetData>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.95780701726897</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.94523872153529</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.14922320741784</v>
+        <v>20.23089785848449</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.25953254286247</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.3139648425288</v>
       </c>
     </row>
   </sheetData>
@@ -4842,13 +4842,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.08930568980784</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.72775465338477</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.93695079176249</v>
+        <v>19.65296630676276</v>
+      </c>
+      <c r="C2" t="n">
+        <v>16.82078466099746</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.98632317929748</v>
       </c>
     </row>
   </sheetData>
@@ -4892,13 +4892,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>18.51411787789205</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.35614157110785</v>
-      </c>
-      <c r="D2" t="n">
-        <v>34.00526830028424</v>
+        <v>16.82653769831421</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.87206693484615</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.02011183374253</v>
       </c>
     </row>
   </sheetData>
@@ -4942,13 +4942,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>23.72334917117123</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.1603842548346</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.14882280839786</v>
+        <v>19.29222156632604</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.30070275939532</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.20540390496978</v>
       </c>
     </row>
   </sheetData>
@@ -4992,13 +4992,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.53046519816744</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.81228479994825</v>
-      </c>
-      <c r="D2" t="n">
-        <v>35.05342748917449</v>
+        <v>21.08662873429117</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.40943466620548</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.03473823191349</v>
       </c>
     </row>
   </sheetData>
@@ -5042,13 +5042,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.72530962866869</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.92471675415169</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.95746773394413</v>
+        <v>21.08293322265116</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.34921088436774</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.82349168349402</v>
       </c>
     </row>
   </sheetData>
@@ -5092,13 +5092,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.44879892648938</v>
-      </c>
-      <c r="C2" t="n">
-        <v>29.89288689695061</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.36112985337611</v>
+        <v>20.94534080430794</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.01910530982525</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.40213381312288</v>
       </c>
     </row>
   </sheetData>
@@ -5142,13 +5142,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.08936745703356</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.09724960237404</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.33440173777834</v>
+        <v>23.53226140620225</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.47564391849057</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.95407811925394</v>
       </c>
     </row>
   </sheetData>
@@ -5192,13 +5192,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.59991587282883</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.40115808607575</v>
-      </c>
-      <c r="D2" t="n">
-        <v>33.83606840785914</v>
+        <v>20.34503044839576</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.48783387451727</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.00435668521073</v>
       </c>
     </row>
   </sheetData>
@@ -5242,13 +5242,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.365224356249</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.76350061281807</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.16523163495244</v>
+        <v>28.22371001144482</v>
+      </c>
+      <c r="C2" t="n">
+        <v>27.30825980163042</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.02553249598864</v>
       </c>
     </row>
   </sheetData>
@@ -5292,13 +5292,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.35032851819323</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.90277169251232</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.46477452280219</v>
+        <v>25.04495445710794</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.58057258557525</v>
+      </c>
+      <c r="D2" t="n">
+        <v>19.05856026591663</v>
       </c>
     </row>
   </sheetData>
@@ -5342,13 +5342,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.23027865296353</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.7421088926628</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.9603607497911</v>
+        <v>17.66663558099425</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.54891749466491</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.06732360608257</v>
       </c>
     </row>
   </sheetData>
@@ -5392,13 +5392,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.96145640040172</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.76943830231313</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.91733380173432</v>
+        <v>24.24888203116561</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.19810499304619</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.38344574496609</v>
       </c>
     </row>
   </sheetData>
@@ -5442,13 +5442,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.91515971286996</v>
-      </c>
-      <c r="C2" t="n">
-        <v>33.80421112538723</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.93070357990063</v>
+        <v>18.46570689182171</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.65117900570561</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.04917088201739</v>
       </c>
     </row>
   </sheetData>
@@ -5492,13 +5492,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>21.98392499894932</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.32626151083153</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.58795806587868</v>
+        <v>19.92601510738172</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.44351918225734</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.59148135795107</v>
       </c>
     </row>
   </sheetData>
@@ -5542,13 +5542,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.00592971409452</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.38405803620814</v>
-      </c>
-      <c r="D2" t="n">
-        <v>35.61096594601325</v>
+        <v>15.01984041894128</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.38564489160334</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.63962374991276</v>
       </c>
     </row>
   </sheetData>
@@ -5592,13 +5592,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.49627078124718</v>
-      </c>
-      <c r="C2" t="n">
-        <v>32.05616125683886</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.12179594359247</v>
+        <v>19.09725991842349</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.93174728731705</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.26424897254456</v>
       </c>
     </row>
   </sheetData>
@@ -5642,13 +5642,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.96200971413042</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.42204574082663</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.36798292818193</v>
+        <v>20.84295014760078</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.03555686430801</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.63422654388857</v>
       </c>
     </row>
   </sheetData>
@@ -5692,13 +5692,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.16508413371342</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.37565127747876</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.73173341065887</v>
+        <v>18.64945107435115</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.27915193956834</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.32396498749132</v>
       </c>
     </row>
   </sheetData>
@@ -5742,13 +5742,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>34.74156170017256</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.40810529695036</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.13383907545784</v>
+        <v>27.0406073121578</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.94975666181343</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.02191474453594</v>
       </c>
     </row>
   </sheetData>
@@ -5792,13 +5792,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.7319921486092</v>
-      </c>
-      <c r="C2" t="n">
-        <v>30.75497357713646</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.80670254293761</v>
+        <v>20.40605762319537</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.92996309106335</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.60168846847741</v>
       </c>
     </row>
   </sheetData>
@@ -5842,13 +5842,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.26387083587054</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.42957198323728</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.78581530708589</v>
+        <v>23.38843646099876</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.78363088913962</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.02019371952326</v>
       </c>
     </row>
   </sheetData>
@@ -5892,13 +5892,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.66950059609909</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.24665346441451</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.61338458094249</v>
+        <v>19.55565588957053</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.14077562863837</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.74612780356495</v>
       </c>
     </row>
   </sheetData>
@@ -5942,13 +5942,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>23.18894283653658</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.59829517877377</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.83901740948378</v>
+        <v>21.17620922403452</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.28789258549509</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.32427967948009</v>
       </c>
     </row>
   </sheetData>
@@ -5992,13 +5992,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.89687520461042</v>
-      </c>
-      <c r="C2" t="n">
-        <v>29.92207285015577</v>
-      </c>
-      <c r="D2" t="n">
-        <v>18.40164678664153</v>
+        <v>22.66886471237598</v>
+      </c>
+      <c r="C2" t="n">
+        <v>17.06340196907843</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.12555933899128</v>
       </c>
     </row>
   </sheetData>
@@ -6042,13 +6042,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.3033819872751</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.12200583434516</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.31541512936245</v>
+        <v>19.91115381182585</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.16737389765959</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.39560617858803</v>
       </c>
     </row>
   </sheetData>
@@ -6092,13 +6092,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.51012064687713</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.54864203465145</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.55177695836077</v>
+        <v>21.06612497760953</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.78407569922085</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.29327798531081</v>
       </c>
     </row>
   </sheetData>
@@ -6142,13 +6142,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.73542259605647</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.02873157160182</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.61250101910888</v>
+        <v>20.48746463560197</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.74898489203786</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.30565869139773</v>
       </c>
     </row>
   </sheetData>
@@ -6192,13 +6192,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.30342772203808</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.74727492486978</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.82021569350095</v>
+        <v>19.24155392424957</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.40974046472162</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.82797950661754</v>
       </c>
     </row>
   </sheetData>
@@ -6242,13 +6242,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.10644669197459</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.55376150661147</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.86617287622672</v>
+        <v>20.58177237052604</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.99908600977782</v>
+      </c>
+      <c r="D2" t="n">
+        <v>31.72665728864947</v>
       </c>
     </row>
   </sheetData>
@@ -6292,13 +6292,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.18284904144188</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.99423351795378</v>
-      </c>
-      <c r="D2" t="n">
-        <v>33.16679070606248</v>
+        <v>20.27802515671529</v>
+      </c>
+      <c r="C2" t="n">
+        <v>27.77966195651588</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.17631635820415</v>
       </c>
     </row>
   </sheetData>
@@ -6342,13 +6342,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.73046144614133</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.63382891395111</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.33820969303554</v>
+        <v>18.62772510257654</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.92805852174351</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.65677825840124</v>
       </c>
     </row>
   </sheetData>
@@ -6392,13 +6392,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.3627033632728</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.004895322379</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.72407711382724</v>
+        <v>21.38189006707753</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.69369126550865</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.91068149946699</v>
       </c>
     </row>
   </sheetData>
@@ -6442,13 +6442,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.79507881987436</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.19671378589848</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.38220775350576</v>
+        <v>26.60678069661711</v>
+      </c>
+      <c r="C2" t="n">
+        <v>27.54332217333995</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.93568833758394</v>
       </c>
     </row>
   </sheetData>
@@ -6492,13 +6492,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.76841337618588</v>
-      </c>
-      <c r="C2" t="n">
-        <v>35.53762415848485</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.80464872185</v>
+        <v>18.41718430835575</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.56309181115533</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.08190724062183</v>
       </c>
     </row>
   </sheetData>
@@ -6542,13 +6542,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.36409315943309</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.22260658815705</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.504430844352</v>
+        <v>23.83125307314965</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.16743748877002</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.11206678451535</v>
       </c>
     </row>
   </sheetData>
@@ -6592,13 +6592,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.73709440112171</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.46585622441958</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.45405431776026</v>
+        <v>18.18907795791355</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.77131087987802</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.8793532604307</v>
       </c>
     </row>
   </sheetData>
@@ -6642,13 +6642,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.36161543482292</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.55538588699985</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.95135202461562</v>
+        <v>19.09380813554425</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.79570934592626</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.01955653999554</v>
       </c>
     </row>
   </sheetData>
@@ -6692,13 +6692,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.68594914332985</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.66583229265814</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.23523472768553</v>
+        <v>19.41224520689848</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.25116742027149</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.88312141531705</v>
       </c>
     </row>
   </sheetData>
@@ -6742,13 +6742,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>23.5561549572117</v>
-      </c>
-      <c r="C2" t="n">
-        <v>31.89178443298761</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.24369904216454</v>
+        <v>24.68784387467281</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.75390799768533</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.98078268758019</v>
       </c>
     </row>
   </sheetData>
@@ -6792,13 +6792,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.09336523027877</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.44347564769833</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.43817997951325</v>
+        <v>17.18431213850956</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.51740573049687</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.96653534826413</v>
       </c>
     </row>
   </sheetData>
@@ -6842,13 +6842,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.51865683167107</v>
-      </c>
-      <c r="C2" t="n">
-        <v>31.21012425816123</v>
-      </c>
-      <c r="D2" t="n">
-        <v>34.86712765528775</v>
+        <v>17.55713479095029</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.06127557399018</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.32151155392437</v>
       </c>
     </row>
   </sheetData>
@@ -6892,13 +6892,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.19786730914388</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.35720854554034</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.24890064294239</v>
+        <v>23.34200399542806</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.24337888961653</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.49706292892946</v>
       </c>
     </row>
   </sheetData>
@@ -6942,13 +6942,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.83109521973631</v>
-      </c>
-      <c r="C2" t="n">
-        <v>30.7001158800176</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.76235843536793</v>
+        <v>24.43295370025422</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.41979438786607</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.00315721555533</v>
       </c>
     </row>
   </sheetData>
@@ -6992,13 +6992,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.18462406011791</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.0314249423125</v>
-      </c>
-      <c r="D2" t="n">
-        <v>36.28223327493148</v>
+        <v>20.62977953255601</v>
+      </c>
+      <c r="C2" t="n">
+        <v>28.58455522662432</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.58903050328047</v>
       </c>
     </row>
   </sheetData>
@@ -7042,13 +7042,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.59033415949766</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.71870056200471</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.42537312891573</v>
+        <v>18.00028347019328</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.77899459391184</v>
+      </c>
+      <c r="D2" t="n">
+        <v>19.54155314419611</v>
       </c>
     </row>
   </sheetData>
@@ -7092,13 +7092,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.08819942028322</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.21818581850279</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.48246096844848</v>
+        <v>23.17802364351613</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.38711327355556</v>
+      </c>
+      <c r="D2" t="n">
+        <v>19.19849653103963</v>
       </c>
     </row>
   </sheetData>
@@ -7142,13 +7142,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.46467884556073</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.49285399184575</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.91356735605867</v>
+        <v>20.79020874858181</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.8763360123302</v>
+      </c>
+      <c r="D2" t="n">
+        <v>29.64035060647061</v>
       </c>
     </row>
   </sheetData>
@@ -7192,13 +7192,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.72820946207831</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.39373315630642</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.96988614234165</v>
+        <v>27.08914176863005</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.37536957006883</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.82014602978568</v>
       </c>
     </row>
   </sheetData>
@@ -7242,13 +7242,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>19.02873957021466</v>
-      </c>
-      <c r="C2" t="n">
-        <v>33.02555919909036</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.26382315236719</v>
+        <v>16.50819186112292</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.1147385442997</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.82861033866125</v>
       </c>
     </row>
   </sheetData>
@@ -7292,13 +7292,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>22.09233683455439</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.31150677800116</v>
-      </c>
-      <c r="D2" t="n">
-        <v>37.75123076796193</v>
+        <v>18.31859281339443</v>
+      </c>
+      <c r="C2" t="n">
+        <v>27.97847481156325</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.18137927754114</v>
       </c>
     </row>
   </sheetData>
@@ -7342,13 +7342,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.5158152082277</v>
-      </c>
-      <c r="C2" t="n">
-        <v>31.66360494812411</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.66324170784545</v>
+        <v>18.77941406791779</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.52206043808184</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.95964305554565</v>
       </c>
     </row>
   </sheetData>
@@ -7392,13 +7392,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.0584939024926</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.35444921213853</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.11694880539275</v>
+        <v>19.03613492298344</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.09340601966469</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.28311098889188</v>
       </c>
     </row>
   </sheetData>
@@ -7442,13 +7442,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.63967678766439</v>
-      </c>
-      <c r="C2" t="n">
-        <v>29.82531353979533</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.82291581988652</v>
+        <v>19.66631609568426</v>
+      </c>
+      <c r="C2" t="n">
+        <v>27.65139887119922</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.29792174903632</v>
       </c>
     </row>
   </sheetData>
@@ -7492,13 +7492,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.93420023043948</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.42588183446052</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.74906889408186</v>
+        <v>25.18832532498334</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.90275421371634</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.95390249283485</v>
       </c>
     </row>
   </sheetData>
@@ -7542,13 +7542,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.20261186501354</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.14544515404483</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.99909049638405</v>
+        <v>18.70660802613432</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.00601856624995</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.81095810709999</v>
       </c>
     </row>
   </sheetData>
@@ -7592,13 +7592,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.31408521150264</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.74857485092133</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.46365827390901</v>
+        <v>19.75702876948419</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24.87278501153757</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.64176263604087</v>
       </c>
     </row>
   </sheetData>
@@ -7642,13 +7642,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>34.48298721658237</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.48723125014835</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.63482475115923</v>
+        <v>17.84152113986404</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24.34289646445907</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.95630343627347</v>
       </c>
     </row>
   </sheetData>
@@ -7692,13 +7692,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.30936555124739</v>
-      </c>
-      <c r="C2" t="n">
-        <v>32.57583508816865</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.57179573450898</v>
+        <v>22.95190386296263</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.03646648117412</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.16618887121192</v>
       </c>
     </row>
   </sheetData>
@@ -7742,13 +7742,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>23.44444623499762</v>
-      </c>
-      <c r="C2" t="n">
-        <v>14.72508936698066</v>
-      </c>
-      <c r="D2" t="n">
-        <v>35.56507799369945</v>
+        <v>22.29402241911286</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.37772070289979</v>
+      </c>
+      <c r="D2" t="n">
+        <v>17.40437097393082</v>
       </c>
     </row>
   </sheetData>
@@ -7792,13 +7792,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>20.80376976506528</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.28530311718316</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.89293458115825</v>
+        <v>20.91677459011696</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.07253230133967</v>
+      </c>
+      <c r="D2" t="n">
+        <v>17.27665842713071</v>
       </c>
     </row>
   </sheetData>
@@ -7842,13 +7842,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.48301289385104</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.74498640744289</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.8763521633646</v>
+        <v>18.68018129430926</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.15350299599178</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.35961616743013</v>
       </c>
     </row>
   </sheetData>
@@ -7892,13 +7892,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.41283845361352</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.19408264457036</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.82843435702108</v>
+        <v>19.30745360618821</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.37457067521473</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.67752134413266</v>
       </c>
     </row>
   </sheetData>
@@ -7942,13 +7942,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.63096648943837</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.00951367632715</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.80709433394701</v>
+        <v>21.51509759740698</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.76286640388281</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.53970882707786</v>
       </c>
     </row>
   </sheetData>
@@ -7992,13 +7992,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.72789121480131</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.43123302338133</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.13102207162143</v>
+        <v>23.28853968204374</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.93363333678308</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.23540915360813</v>
       </c>
     </row>
   </sheetData>
@@ -8042,13 +8042,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.74105527828652</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.44625850581516</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.11991682367882</v>
+        <v>18.16912604203361</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.3159966302766</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.1668152256101</v>
       </c>
     </row>
   </sheetData>
@@ -8092,13 +8092,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.21417997639984</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.18885931603759</v>
-      </c>
-      <c r="D2" t="n">
-        <v>33.13508689317036</v>
+        <v>23.89008305338607</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.49912625448871</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.18652893867061</v>
       </c>
     </row>
   </sheetData>
@@ -8142,13 +8142,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.85112949119004</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.18947409781581</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.22631181383436</v>
+        <v>17.37846082251379</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.71377037648277</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.87420352611479</v>
       </c>
     </row>
   </sheetData>
@@ -8192,13 +8192,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.38104537083225</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.98067585593383</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.84749629893379</v>
+        <v>20.25185761575083</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.35049349526711</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.6219900656521</v>
       </c>
     </row>
   </sheetData>
@@ -8242,13 +8242,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.45377456929072</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.73563844310345</v>
-      </c>
-      <c r="D2" t="n">
-        <v>33.54969679118632</v>
+        <v>20.21821691838957</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.71718358992914</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.89571416088433</v>
       </c>
     </row>
   </sheetData>
@@ -8292,13 +8292,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.23177184723438</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.10611132045815</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.47871035805099</v>
+        <v>22.29837340125731</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.49059768713598</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.35944855206496</v>
       </c>
     </row>
   </sheetData>
@@ -8342,13 +8342,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>21.38179911030743</v>
-      </c>
-      <c r="C2" t="n">
-        <v>34.66495564060308</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.99594790066578</v>
+        <v>19.21792560191299</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.35094727281337</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.21331301752042</v>
       </c>
     </row>
   </sheetData>
@@ -8392,13 +8392,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.53217106917584</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.48556389160781</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.65541377492025</v>
+        <v>17.86151915098231</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.9970074638257</v>
+      </c>
+      <c r="D2" t="n">
+        <v>18.73293450260856</v>
       </c>
     </row>
   </sheetData>
@@ -8442,13 +8442,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.31648799767439</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.42366469142474</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.97558312765094</v>
+        <v>20.14618056291231</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.81693738383894</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.42327277957905</v>
       </c>
     </row>
   </sheetData>
@@ -8492,13 +8492,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>34.54800191020548</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.50821452371563</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.44589819128782</v>
+        <v>20.03638439588645</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.04406901363239</v>
+      </c>
+      <c r="D2" t="n">
+        <v>29.02493243212789</v>
       </c>
     </row>
   </sheetData>
@@ -8542,13 +8542,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>20.09998403884269</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.6176907987473</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.24183434186633</v>
+        <v>18.12426751951305</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.52509684147509</v>
+      </c>
+      <c r="D2" t="n">
+        <v>18.95701549287211</v>
       </c>
     </row>
   </sheetData>
@@ -8592,13 +8592,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.55081026534635</v>
-      </c>
-      <c r="C2" t="n">
-        <v>29.67428189442034</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.16578442708409</v>
+        <v>25.77280973337545</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.18014623289976</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.00770230296507</v>
       </c>
     </row>
   </sheetData>
@@ -8642,13 +8642,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.2483986105011</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.22553534250263</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.0840027573865</v>
+        <v>18.25813170776703</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.52205297098083</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26.45073546548296</v>
       </c>
     </row>
   </sheetData>
@@ -8692,13 +8692,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.59778752576444</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.37436081096494</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.94585207489834</v>
+        <v>18.66233939315821</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.22774070395864</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.11056433939066</v>
       </c>
     </row>
   </sheetData>
@@ -8742,13 +8742,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.41479618479542</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.62895040811953</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.80999478498221</v>
+        <v>25.50661027011892</v>
+      </c>
+      <c r="C2" t="n">
+        <v>32.20780342110491</v>
+      </c>
+      <c r="D2" t="n">
+        <v>19.9157365519017</v>
       </c>
     </row>
   </sheetData>
@@ -8792,13 +8792,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.27326067434666</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.19114899542105</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.99047438609009</v>
+        <v>23.1762330268907</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.14453951271887</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.62746829815487</v>
       </c>
     </row>
   </sheetData>
@@ -8842,13 +8842,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.28181491748935</v>
-      </c>
-      <c r="C2" t="n">
-        <v>30.15515937002354</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.84047147184727</v>
+        <v>21.69096377632725</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.66494523807498</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.86329606015087</v>
       </c>
     </row>
   </sheetData>
@@ -8892,13 +8892,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.34995688551026</v>
-      </c>
-      <c r="C2" t="n">
-        <v>32.14012469620555</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.46911447740827</v>
+        <v>18.11550043174823</v>
+      </c>
+      <c r="C2" t="n">
+        <v>28.64422600398576</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.53135297231751</v>
       </c>
     </row>
   </sheetData>
@@ -8942,13 +8942,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.5210218688459</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.86473352654489</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.58789417388856</v>
+        <v>18.66970596744362</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.97456535866329</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.03163031641209</v>
       </c>
     </row>
   </sheetData>
@@ -8992,13 +8992,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>22.68295249732611</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.63393603831371</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.06107287516288</v>
+        <v>16.58427262952565</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.55329819149009</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.26497684966367</v>
       </c>
     </row>
   </sheetData>
@@ -9042,13 +9042,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.84782544686434</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.02548004348037</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.10951011919077</v>
+        <v>23.06250099608088</v>
+      </c>
+      <c r="C2" t="n">
+        <v>27.92554791704165</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.9926738737196</v>
       </c>
     </row>
   </sheetData>
@@ -9092,13 +9092,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>23.52972175517225</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.0990395132652</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.3880081689548</v>
+        <v>18.83760979962302</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.62709687454529</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.28327243707647</v>
       </c>
     </row>
   </sheetData>
@@ -9142,13 +9142,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.67933147653255</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.43614287874326</v>
-      </c>
-      <c r="D2" t="n">
-        <v>34.39433710558048</v>
+        <v>21.10402479677138</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.59130145641136</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.8080285758173</v>
       </c>
     </row>
   </sheetData>
@@ -9192,13 +9192,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.69754471552891</v>
-      </c>
-      <c r="C2" t="n">
-        <v>34.64552167426959</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.78935038252293</v>
+        <v>21.42463739084916</v>
+      </c>
+      <c r="C2" t="n">
+        <v>28.93541736605686</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.56151607671166</v>
       </c>
     </row>
   </sheetData>
@@ -9242,13 +9242,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.26489675321843</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.57985330777584</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.03176076109498</v>
+        <v>18.79764675002102</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.95641604890854</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.79091350696433</v>
       </c>
     </row>
   </sheetData>
@@ -9292,13 +9292,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.19626924792643</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.28479094499445</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.36574290656381</v>
+        <v>19.1249071308066</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.73819955878229</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.41376309662715</v>
       </c>
     </row>
   </sheetData>
@@ -9342,13 +9342,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.33736347570808</v>
-      </c>
-      <c r="C2" t="n">
-        <v>33.54918890534846</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.18772591181732</v>
+        <v>25.43892505626168</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.99669221316107</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.917619185075</v>
       </c>
     </row>
   </sheetData>
@@ -9392,13 +9392,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>32.9389787971248</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.73089945971169</v>
-      </c>
-      <c r="D2" t="n">
-        <v>38.20937779766537</v>
+        <v>20.2806696055982</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.92808438009735</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.43412090033671</v>
       </c>
     </row>
   </sheetData>
@@ -9442,13 +9442,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.7418260192681</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.32429950891461</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.01733733796842</v>
+        <v>19.81640902718211</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.07964143137731</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.39615432765479</v>
       </c>
     </row>
   </sheetData>
@@ -9492,13 +9492,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.8860294616693</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.19747246501421</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.34763683850856</v>
+        <v>19.11819776680957</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.03256780024597</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.42829991285216</v>
       </c>
     </row>
   </sheetData>
@@ -9542,13 +9542,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>33.50706509316328</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.07496309434811</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30.9276127037743</v>
+        <v>23.52453813473173</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.09817817358969</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.15320831555184</v>
       </c>
     </row>
   </sheetData>
@@ -9592,13 +9592,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>33.34099072701799</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.97340887382689</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32.02904506321394</v>
+        <v>23.33765225921457</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.43306539009231</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.82376765587544</v>
       </c>
     </row>
   </sheetData>
@@ -9642,13 +9642,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>35.09400056627361</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.70812154956989</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.61081746460752</v>
+        <v>24.37806611636798</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.77820724034018</v>
+      </c>
+      <c r="D2" t="n">
+        <v>29.04964443811878</v>
       </c>
     </row>
   </sheetData>
@@ -9692,13 +9692,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>21.11342624035067</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.26382834209543</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.70826548087035</v>
+        <v>19.84890446384956</v>
+      </c>
+      <c r="C2" t="n">
+        <v>26.85092134745066</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.15515722788284</v>
       </c>
     </row>
   </sheetData>
@@ -9742,13 +9742,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.06563614235044</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.90653217318517</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.59606749980162</v>
+        <v>23.82800750387396</v>
+      </c>
+      <c r="C2" t="n">
+        <v>14.62332098003935</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.64465044642884</v>
       </c>
     </row>
   </sheetData>
@@ -9792,13 +9792,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.42152263214249</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.55693696388679</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.01330275620741</v>
+        <v>18.49621260240595</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.42400718646268</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.12703835232413</v>
       </c>
     </row>
   </sheetData>
@@ -9842,13 +9842,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>23.42435880207744</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.72165141640378</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.83767745142251</v>
+        <v>15.80455647861453</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.21338820770614</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.83827318697061</v>
       </c>
     </row>
   </sheetData>
@@ -9892,13 +9892,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>22.84398245318509</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.29407563412094</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.57668991263499</v>
+        <v>20.07385424992928</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24.10887600299875</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.61696758660021</v>
       </c>
     </row>
   </sheetData>
@@ -9942,13 +9942,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>35.66631015348404</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.6384864383167</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.57934080228413</v>
+        <v>20.62993308642147</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.45801806132866</v>
+      </c>
+      <c r="D2" t="n">
+        <v>17.08342917639991</v>
       </c>
     </row>
   </sheetData>
@@ -9992,13 +9992,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>27.1239665255933</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.0523497940352</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.52347173764035</v>
+        <v>18.2720850891397</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.35699832048771</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.44722938413592</v>
       </c>
     </row>
   </sheetData>
@@ -10042,13 +10042,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>31.19045131334382</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.62303454831343</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.3128298121612</v>
+        <v>27.92429675082286</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.87960552515594</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.04593619715587</v>
       </c>
     </row>
   </sheetData>
@@ -10092,13 +10092,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>33.22876797487366</v>
-      </c>
-      <c r="C2" t="n">
-        <v>33.51731919955206</v>
-      </c>
-      <c r="D2" t="n">
-        <v>20.72295077630572</v>
+        <v>15.73342097094839</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25.08841397550784</v>
+      </c>
+      <c r="D2" t="n">
+        <v>27.41844528522946</v>
       </c>
     </row>
   </sheetData>
@@ -10142,13 +10142,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.86620065900053</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.90255424595032</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.31809846423743</v>
+        <v>19.84758656484168</v>
+      </c>
+      <c r="C2" t="n">
+        <v>28.07550475109457</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20.89490821521093</v>
       </c>
     </row>
   </sheetData>
@@ -10192,13 +10192,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>25.88923641155149</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.21582042403217</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.837142057713</v>
+        <v>22.79480311036295</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.50578046485725</v>
+      </c>
+      <c r="D2" t="n">
+        <v>19.99128259366315</v>
       </c>
     </row>
   </sheetData>
@@ -10242,13 +10242,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.32090985244281</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.39087562166305</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.94426079636484</v>
+        <v>29.31804506045219</v>
+      </c>
+      <c r="C2" t="n">
+        <v>18.05785198720015</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.28669305715586</v>
       </c>
     </row>
   </sheetData>
@@ -10292,13 +10292,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>36.26761709478797</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.20935177031887</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.72025875118634</v>
+        <v>23.5524929718785</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.55037960398354</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25.3299765695464</v>
       </c>
     </row>
   </sheetData>
@@ -10342,13 +10342,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>26.08560210945038</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.54826840546856</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.00204866005659</v>
+        <v>25.07761843202305</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21.25643493319888</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.92810899418152</v>
       </c>
     </row>
   </sheetData>
@@ -10392,13 +10392,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>23.35578882568737</v>
-      </c>
-      <c r="C2" t="n">
-        <v>32.21262916305475</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.66138218525813</v>
+        <v>20.9209002158592</v>
+      </c>
+      <c r="C2" t="n">
+        <v>30.59498679868985</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.86973123670533</v>
       </c>
     </row>
   </sheetData>
@@ -10442,13 +10442,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>30.55789517621375</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.54559375512889</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.54184933434984</v>
+        <v>17.67157627765875</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.60344025671011</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24.18267858437782</v>
       </c>
     </row>
   </sheetData>
@@ -10492,13 +10492,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>29.36494038365652</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.50287728926058</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.54803388066104</v>
+        <v>19.2016680142622</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19.87517254994919</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.70925150658866</v>
       </c>
     </row>
   </sheetData>
@@ -10542,13 +10542,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>22.49429460422881</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.13221870645768</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.02552280324668</v>
+        <v>21.09968604794853</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.76703432479522</v>
+      </c>
+      <c r="D2" t="n">
+        <v>19.58675441082478</v>
       </c>
     </row>
   </sheetData>
@@ -10592,13 +10592,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>28.24401865451406</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.91952642465924</v>
-      </c>
-      <c r="D2" t="n">
-        <v>31.44538793508013</v>
+        <v>19.2250740395055</v>
+      </c>
+      <c r="C2" t="n">
+        <v>27.1355855227999</v>
+      </c>
+      <c r="D2" t="n">
+        <v>28.65681116674646</v>
       </c>
     </row>
   </sheetData>

</xml_diff>